<commit_message>
Valuta steg 3: försäljning i valuta — kund, prislista, kundorder, faktura och kundbetalning i valuta
Kunder och prislistor får valuta, kundordern snapshotar valuta och kurs och
prissätter särpris i kundens valuta, prislista i orderns valuta och
artikelpriset omräknat. Kundfakturan tar kursen vid Utfärda (eller en manuell
kurs), kreditfakturan källfakturans kurs, och bokförs i SEK med restmetoden.
Kundbetalningen bokför frigjort SEK, insatt SEK-belopp, bankavgift och
kursvinst/-förlust; camt.054-kredit med InstdAmt i fakturans valuta matchas
och bokförs med postens SEK-belopp. Samlingsfakturering per kund och valuta,
påminnelseavgift bara i SEK, rapporterna räknar om till SEK, konfiguratorns
evaluate tar valuta. Kundimportens Valuta och importmallen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015RSdtiEAvRGDcuA9MaSsvt
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-kunder.xlsx
+++ b/apps/web/public/importmallar/importmall-kunder.xlsx
@@ -383,6 +383,18 @@
             <family val="2"/>
           </rPr>
           <t xml:space="preserve">Max 255 tecken. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Valutakod med tre bokstäver (SEK, EUR, NOK …); små bokstäver godtas, annat ger ett fel. Nya offerter och kundordrar får kundens valuta och dagens kurs, och kundens kundpriser gäller i den valutan; befintliga ordrar behåller sin. Tom cell ger SEK för nya kunder och lämnar befintliga orörda.</t>
         </r>
       </text>
     </comment>
@@ -477,6 +489,7 @@
     <col min="29" max="29" width="19" customWidth="1"/>
     <col min="30" max="30" width="16" customWidth="1"/>
     <col min="31" max="31" width="14" customWidth="1"/>
+    <col min="32" max="32" width="14" customWidth="1" style="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -633,6 +646,11 @@
       <c r="AE1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Webbsida</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valuta</t>
         </is>
       </c>
     </row>
@@ -1392,6 +1410,28 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valuta</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Valutakod med tre bokstäver (SEK, EUR, NOK …); små bokstäver godtas, annat ger ett fel. Nya offerter och kundordrar får kundens valuta och dagens kurs, och kundens kundpriser gäller i den valutan; befintliga ordrar behåller sin. Tom cell ger SEK för nya kunder och lämnar befintliga orörda.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEK</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Faktura i vänteläge på kunden
customers.invoice_on_hold (0165): kundens fakturor granskas före utskick. Samlingsfaktureringens Utfärda direkt lämnar kundens faktura som utkast (resultatraden "Utkast — Faktura i vänteläge"), fakturakortet påminner på utkastet, manuell Utfärda fungerar som vanligt. Kryssruta på kundkortet och kundimportens kolumn Faktura i vänteläge.

Hela API-sviten grön (6568); etapp 3 (Kalkylpris 2, Säkerhetslager/Styrning, Transportkostnad, Faktura i vänteläge) kontrollerad i Chromium, även i mobilbredd.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013pvWaFZiioxpDd9AVeYPCR
</commit_message>
<xml_diff>
--- a/apps/web/public/importmallar/importmall-kunder.xlsx
+++ b/apps/web/public/importmallar/importmall-kunder.xlsx
@@ -370,11 +370,23 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja betyder att kundens fakturor granskas före utskick: samlingsfaktureringens Utfärda direkt lämnar dem som utkast. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
           <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja visar priser inklusive moms på kundens offerter, orderbekräftelser och fakturor. Tom cell lämnar fältet orört på en befintlig post.</t>
         </r>
       </text>
     </comment>
-    <comment ref="AE1" authorId="0">
+    <comment ref="AF1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -386,7 +398,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF1" authorId="0">
+    <comment ref="AG1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -487,9 +499,10 @@
     <col min="27" max="27" width="22" customWidth="1"/>
     <col min="28" max="28" width="26" customWidth="1" style="4"/>
     <col min="29" max="29" width="19" customWidth="1"/>
-    <col min="30" max="30" width="16" customWidth="1"/>
-    <col min="31" max="31" width="14" customWidth="1"/>
-    <col min="32" max="32" width="14" customWidth="1" style="4"/>
+    <col min="30" max="30" width="23" customWidth="1"/>
+    <col min="31" max="31" width="16" customWidth="1"/>
+    <col min="32" max="32" width="14" customWidth="1"/>
+    <col min="33" max="33" width="14" customWidth="1" style="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -640,15 +653,20 @@
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Faktura i vänteläge</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Privatperson</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Webbsida</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Valuta</t>
         </is>
@@ -1369,7 +1387,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Privatperson</t>
+          <t xml:space="preserve">Faktura i vänteläge</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -1379,7 +1397,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja visar priser inklusive moms på kundens offerter, orderbekräftelser och fakturor. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja betyder att kundens fakturor granskas före utskick: samlingsfaktureringens Utfärda direkt lämnar dem som utkast. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1391,7 +1409,7 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Webbsida</t>
+          <t xml:space="preserve">Privatperson</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -1401,32 +1419,54 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Max 255 tecken. Tom cell lämnar fältet orört på en befintlig post.</t>
+          <t xml:space="preserve">Ja/Nej, 1/0, X eller true/false — Ja visar priser inklusive moms på kundens offerter, orderbekräftelser och fakturor. Tom cell lämnar fältet orört på en befintlig post.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.example.com</t>
+          <t xml:space="preserve">Nej</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Webbsida</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max 255 tecken. Tom cell lämnar fältet orört på en befintlig post.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Valuta</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nej</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nej</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Valutakod med tre bokstäver (SEK, EUR, NOK …); små bokstäver godtas, annat ger ett fel. Nya offerter och kundordrar får kundens valuta och dagens kurs, och kundens kundpriser gäller i den valutan; befintliga ordrar behåller sin. Tom cell ger SEK för nya kunder och lämnar befintliga orörda.</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">SEK</t>
         </is>

</xml_diff>